<commit_message>
Add KPIX contacts: Hannah Blazei + assignment editors DL
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L2766C7NnASe5xwMeG2Sg2
</commit_message>
<xml_diff>
--- a/files/BHU_Master_Press_List.xlsx
+++ b/files/BHU_Master_Press_List.xlsx
@@ -423,14 +423,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I111"/>
+  <dimension ref="A1:I113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
@@ -440,7 +440,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MASTER PRESS LIST — updated after Jul 14 2026 press release</t>
+          <t>MASTER PRESS LIST — updated 2026-07-14</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -455,7 +455,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>107 contacts · 8 hard bounces removed Jul 14 (moved to Removed tab)</t>
+          <t>109 contacts · bounces removed Jul 14 · KPIX contacts added Jul 14</t>
         </is>
       </c>
       <c r="B2" s="1" t="n"/>
@@ -2249,7 +2249,11 @@
       <c r="I57" s="1" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n"/>
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>Hannah Blazei</t>
+        </is>
+      </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
           <t>KPIX / CBS Bay Area</t>
@@ -2257,124 +2261,124 @@
       </c>
       <c r="C58" s="1" t="inlineStr">
         <is>
-          <t>newsdesk@kpix.com</t>
+          <t>hannah.blazei@cbs.com</t>
         </is>
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t>News desk / general</t>
+          <t>Reporter / journalist</t>
         </is>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>Not yet verified</t>
+          <t>added manually Jul 14 2026 (user contact)</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>TV general assignment (inferred — verify)</t>
-        </is>
-      </c>
-      <c r="G58" s="1" t="inlineStr">
-        <is>
-          <t>415- 954-7321</t>
-        </is>
-      </c>
+          <t>KPIX assignment desk / Bay Area news</t>
+        </is>
+      </c>
+      <c r="G58" s="1" t="n"/>
       <c r="H58" s="1" t="n"/>
       <c r="I58" s="1" t="inlineStr">
         <is>
-          <t>MED — CBS Bay Area desk</t>
+          <t>HIGH — direct KPIX contact</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>Sara Hossaini</t>
+          <t>KPIX News Assignment Editors (CBS DL)</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
-          <t>KQED</t>
+          <t>KPIX / CBS Bay Area</t>
         </is>
       </c>
       <c r="C59" s="1" t="inlineStr">
         <is>
-          <t>shossaini@kqed.org</t>
+          <t>lcdl_kpixnewsassign.editors@paramount.com</t>
         </is>
       </c>
       <c r="D59" s="1" t="inlineStr">
         <is>
-          <t>Reporter / journalist</t>
+          <t>News desk / general</t>
         </is>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>Not yet verified</t>
+          <t>added manually Jul 14 2026 (user contact)</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>Public radio/TV news (inferred — verify)</t>
+          <t>KPIX assignment desk distribution list</t>
         </is>
       </c>
       <c r="G59" s="1" t="n"/>
       <c r="H59" s="1" t="n"/>
       <c r="I59" s="1" t="inlineStr">
         <is>
-          <t>MED — KQED</t>
+          <t>HIGH — reaches all KPIX assignment editors</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="inlineStr">
-        <is>
-          <t>Vanessa Rancano</t>
-        </is>
-      </c>
+      <c r="A60" s="1" t="n"/>
       <c r="B60" s="1" t="inlineStr">
         <is>
+          <t>KPIX / CBS Bay Area</t>
+        </is>
+      </c>
+      <c r="C60" s="1" t="inlineStr">
+        <is>
+          <t>newsdesk@kpix.com</t>
+        </is>
+      </c>
+      <c r="D60" s="1" t="inlineStr">
+        <is>
+          <t>News desk / general</t>
+        </is>
+      </c>
+      <c r="E60" s="1" t="inlineStr">
+        <is>
+          <t>Not yet verified</t>
+        </is>
+      </c>
+      <c r="F60" s="1" t="inlineStr">
+        <is>
+          <t>TV general assignment (inferred — verify)</t>
+        </is>
+      </c>
+      <c r="G60" s="1" t="inlineStr">
+        <is>
+          <t>415- 954-7321</t>
+        </is>
+      </c>
+      <c r="H60" s="1" t="n"/>
+      <c r="I60" s="1" t="inlineStr">
+        <is>
+          <t>MED — CBS Bay Area desk</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t>Sara Hossaini</t>
+        </is>
+      </c>
+      <c r="B61" s="1" t="inlineStr">
+        <is>
           <t>KQED</t>
         </is>
       </c>
-      <c r="C60" s="1" t="inlineStr">
-        <is>
-          <t>vrancano@kqed.org</t>
-        </is>
-      </c>
-      <c r="D60" s="1" t="inlineStr">
-        <is>
-          <t>Reporter / journalist</t>
-        </is>
-      </c>
-      <c r="E60" s="1" t="inlineStr">
-        <is>
-          <t>Not yet verified</t>
-        </is>
-      </c>
-      <c r="F60" s="1" t="inlineStr">
-        <is>
-          <t>Public radio/TV news (inferred — verify)</t>
-        </is>
-      </c>
-      <c r="G60" s="1" t="n"/>
-      <c r="H60" s="1" t="inlineStr">
-        <is>
-          <t>Inbox full on Mar 5 — valid, resend OK</t>
-        </is>
-      </c>
-      <c r="I60" s="1" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="1" t="n"/>
-      <c r="B61" s="1" t="inlineStr">
-        <is>
-          <t>KQED</t>
-        </is>
-      </c>
       <c r="C61" s="1" t="inlineStr">
         <is>
-          <t>aemslie@kqed.org</t>
+          <t>shossaini@kqed.org</t>
         </is>
       </c>
       <c r="D61" s="1" t="inlineStr">
@@ -2394,22 +2398,26 @@
       </c>
       <c r="G61" s="1" t="n"/>
       <c r="H61" s="1" t="n"/>
-      <c r="I61" s="1" t="n"/>
+      <c r="I61" s="1" t="inlineStr">
+        <is>
+          <t>MED — KQED</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>Sara Stinson</t>
+          <t>Vanessa Rancano</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
-          <t>KRON4</t>
+          <t>KQED</t>
         </is>
       </c>
       <c r="C62" s="1" t="inlineStr">
         <is>
-          <t>sstinson@kron4.com</t>
+          <t>vrancano@kqed.org</t>
         </is>
       </c>
       <c r="D62" s="1" t="inlineStr">
@@ -2419,18 +2427,18 @@
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>ACTIVE (verified)</t>
+          <t>Not yet verified</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>Bay Area general assignment — crime, local government, community/human-interest; covers Oakland &amp; Berkeley</t>
+          <t>Public radio/TV news (inferred — verify)</t>
         </is>
       </c>
       <c r="G62" s="1" t="n"/>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>Verify: a same-name reporter surfaced at CBS New York — KRON4 bylines through Apr 2026 say she's still here</t>
+          <t>Inbox full on Mar 5 — valid, resend OK</t>
         </is>
       </c>
       <c r="I62" s="1" t="n"/>
@@ -2439,17 +2447,17 @@
       <c r="A63" s="1" t="n"/>
       <c r="B63" s="1" t="inlineStr">
         <is>
-          <t>KRON4</t>
+          <t>KQED</t>
         </is>
       </c>
       <c r="C63" s="1" t="inlineStr">
         <is>
-          <t>assignmentdesk@kron.com</t>
+          <t>aemslie@kqed.org</t>
         </is>
       </c>
       <c r="D63" s="1" t="inlineStr">
         <is>
-          <t>News desk / general</t>
+          <t>Reporter / journalist</t>
         </is>
       </c>
       <c r="E63" s="1" t="inlineStr">
@@ -2459,35 +2467,27 @@
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>TV general assignment (inferred — verify)</t>
-        </is>
-      </c>
-      <c r="G63" s="1" t="inlineStr">
-        <is>
-          <t>1 (800) 678-3375</t>
-        </is>
-      </c>
+          <t>Public radio/TV news (inferred — verify)</t>
+        </is>
+      </c>
+      <c r="G63" s="1" t="n"/>
       <c r="H63" s="1" t="n"/>
-      <c r="I63" s="1" t="inlineStr">
-        <is>
-          <t>MED — KRON4 desk</t>
-        </is>
-      </c>
+      <c r="I63" s="1" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>Benjamin Oreskes</t>
+          <t>Sara Stinson</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
-          <t>Los Angeles Times</t>
+          <t>KRON4</t>
         </is>
       </c>
       <c r="C64" s="1" t="inlineStr">
         <is>
-          <t>benjamin.oreskes@latimes.com</t>
+          <t>sstinson@kron4.com</t>
         </is>
       </c>
       <c r="D64" s="1" t="inlineStr">
@@ -2497,37 +2497,37 @@
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>Not yet verified</t>
+          <t>ACTIVE (verified)</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>California news (inferred — verify)</t>
+          <t>Bay Area general assignment — crime, local government, community/human-interest; covers Oakland &amp; Berkeley</t>
         </is>
       </c>
       <c r="G64" s="1" t="n"/>
-      <c r="H64" s="1" t="n"/>
+      <c r="H64" s="1" t="inlineStr">
+        <is>
+          <t>Verify: a same-name reporter surfaced at CBS New York — KRON4 bylines through Apr 2026 say she's still here</t>
+        </is>
+      </c>
       <c r="I64" s="1" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="inlineStr">
-        <is>
-          <t>Susan Rust</t>
-        </is>
-      </c>
+      <c r="A65" s="1" t="n"/>
       <c r="B65" s="1" t="inlineStr">
         <is>
-          <t>Los Angeles Times</t>
+          <t>KRON4</t>
         </is>
       </c>
       <c r="C65" s="1" t="inlineStr">
         <is>
-          <t>susan.rust@latimes.com</t>
+          <t>assignmentdesk@kron.com</t>
         </is>
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t>Reporter / journalist</t>
+          <t>News desk / general</t>
         </is>
       </c>
       <c r="E65" s="1" t="inlineStr">
@@ -2537,27 +2537,35 @@
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>California news (inferred — verify)</t>
-        </is>
-      </c>
-      <c r="G65" s="1" t="n"/>
+          <t>TV general assignment (inferred — verify)</t>
+        </is>
+      </c>
+      <c r="G65" s="1" t="inlineStr">
+        <is>
+          <t>1 (800) 678-3375</t>
+        </is>
+      </c>
       <c r="H65" s="1" t="n"/>
-      <c r="I65" s="1" t="n"/>
+      <c r="I65" s="1" t="inlineStr">
+        <is>
+          <t>MED — KRON4 desk</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>Adrian Rodriguez</t>
+          <t>Benjamin Oreskes</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
-          <t>Marin Independent Journal</t>
+          <t>Los Angeles Times</t>
         </is>
       </c>
       <c r="C66" s="1" t="inlineStr">
         <is>
-          <t>arodriguez@marinij.com</t>
+          <t>benjamin.oreskes@latimes.com</t>
         </is>
       </c>
       <c r="D66" s="1" t="inlineStr">
@@ -2572,7 +2580,7 @@
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>Marin County local news (inferred — verify)</t>
+          <t>California news (inferred — verify)</t>
         </is>
       </c>
       <c r="G66" s="1" t="n"/>
@@ -2582,17 +2590,17 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>Alex Gencan</t>
+          <t>Susan Rust</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t>Marin Independent Journal</t>
+          <t>Los Angeles Times</t>
         </is>
       </c>
       <c r="C67" s="1" t="inlineStr">
         <is>
-          <t>agenca@marinij.com</t>
+          <t>susan.rust@latimes.com</t>
         </is>
       </c>
       <c r="D67" s="1" t="inlineStr">
@@ -2607,7 +2615,7 @@
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>Marin County local news (inferred — verify)</t>
+          <t>California news (inferred — verify)</t>
         </is>
       </c>
       <c r="G67" s="1" t="n"/>
@@ -2617,7 +2625,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>C. MacDonald</t>
+          <t>Adrian Rodriguez</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2627,7 +2635,7 @@
       </c>
       <c r="C68" s="1" t="inlineStr">
         <is>
-          <t>cmacdonald@marinij.com</t>
+          <t>arodriguez@marinij.com</t>
         </is>
       </c>
       <c r="D68" s="1" t="inlineStr">
@@ -2652,7 +2660,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>Dave Allen</t>
+          <t>Alex Gencan</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2662,7 +2670,7 @@
       </c>
       <c r="C69" s="1" t="inlineStr">
         <is>
-          <t>dallen@marinij.com</t>
+          <t>agenca@marinij.com</t>
         </is>
       </c>
       <c r="D69" s="1" t="inlineStr">
@@ -2687,7 +2695,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>G. Klien</t>
+          <t>C. MacDonald</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2697,7 +2705,7 @@
       </c>
       <c r="C70" s="1" t="inlineStr">
         <is>
-          <t>gklien@marinij.com</t>
+          <t>cmacdonald@marinij.com</t>
         </is>
       </c>
       <c r="D70" s="1" t="inlineStr">
@@ -2722,7 +2730,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>Richard Halstead</t>
+          <t>Dave Allen</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2732,7 +2740,7 @@
       </c>
       <c r="C71" s="1" t="inlineStr">
         <is>
-          <t>rhalstead@marinij.com</t>
+          <t>dallen@marinij.com</t>
         </is>
       </c>
       <c r="D71" s="1" t="inlineStr">
@@ -2757,7 +2765,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>S. Rosenfeld</t>
+          <t>G. Klien</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2767,7 +2775,7 @@
       </c>
       <c r="C72" s="1" t="inlineStr">
         <is>
-          <t>srosenfeld@marinij.com</t>
+          <t>gklien@marinij.com</t>
         </is>
       </c>
       <c r="D72" s="1" t="inlineStr">
@@ -2790,20 +2798,24 @@
       <c r="I72" s="1" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n"/>
+      <c r="A73" s="1" t="inlineStr">
+        <is>
+          <t>Richard Halstead</t>
+        </is>
+      </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
-          <t>NBC Bay Area</t>
+          <t>Marin Independent Journal</t>
         </is>
       </c>
       <c r="C73" s="1" t="inlineStr">
         <is>
-          <t>newstips@nbcbayarea.com</t>
+          <t>rhalstead@marinij.com</t>
         </is>
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t>News desk / general</t>
+          <t>Reporter / journalist</t>
         </is>
       </c>
       <c r="E73" s="1" t="inlineStr">
@@ -2813,35 +2825,27 @@
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>TV general assignment (inferred — verify)</t>
-        </is>
-      </c>
-      <c r="G73" s="1" t="inlineStr">
-        <is>
-          <t>1 (408) 432-4780</t>
-        </is>
-      </c>
+          <t>Marin County local news (inferred — verify)</t>
+        </is>
+      </c>
+      <c r="G73" s="1" t="n"/>
       <c r="H73" s="1" t="n"/>
-      <c r="I73" s="1" t="inlineStr">
-        <is>
-          <t>MED — regional TV desk</t>
-        </is>
-      </c>
+      <c r="I73" s="1" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>Bita Ryan</t>
+          <t>S. Rosenfeld</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t>NBC Bay Area / NBCUniversal</t>
+          <t>Marin Independent Journal</t>
         </is>
       </c>
       <c r="C74" s="1" t="inlineStr">
         <is>
-          <t>bita.ryan@nbcuni.com</t>
+          <t>srosenfeld@marinij.com</t>
         </is>
       </c>
       <c r="D74" s="1" t="inlineStr">
@@ -2856,7 +2860,7 @@
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>TV news (inferred — verify)</t>
+          <t>Marin County local news (inferred — verify)</t>
         </is>
       </c>
       <c r="G74" s="1" t="n"/>
@@ -2864,24 +2868,20 @@
       <c r="I74" s="1" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="inlineStr">
-        <is>
-          <t>Velena Jones</t>
-        </is>
-      </c>
+      <c r="A75" s="1" t="n"/>
       <c r="B75" s="1" t="inlineStr">
         <is>
-          <t>NBC Bay Area / NBCUniversal</t>
+          <t>NBC Bay Area</t>
         </is>
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t>velena.jones@nbcuni.com</t>
+          <t>newstips@nbcbayarea.com</t>
         </is>
       </c>
       <c r="D75" s="1" t="inlineStr">
         <is>
-          <t>Reporter / journalist</t>
+          <t>News desk / general</t>
         </is>
       </c>
       <c r="E75" s="1" t="inlineStr">
@@ -2891,35 +2891,35 @@
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>TV news (inferred — verify)</t>
-        </is>
-      </c>
-      <c r="G75" s="1" t="n"/>
-      <c r="H75" s="1" t="inlineStr">
-        <is>
-          <t>Typo variant nbcunic.com bounced Mar 5 — verify spelling</t>
-        </is>
-      </c>
+          <t>TV general assignment (inferred — verify)</t>
+        </is>
+      </c>
+      <c r="G75" s="1" t="inlineStr">
+        <is>
+          <t>1 (408) 432-4780</t>
+        </is>
+      </c>
+      <c r="H75" s="1" t="n"/>
       <c r="I75" s="1" t="inlineStr">
         <is>
-          <t>MED — NBC Bay Area reporter</t>
+          <t>MED — regional TV desk</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>Paul Swensen</t>
+          <t>Bita Ryan</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
         <is>
-          <t>NorCal Public Media</t>
+          <t>NBC Bay Area / NBCUniversal</t>
         </is>
       </c>
       <c r="C76" s="1" t="inlineStr">
         <is>
-          <t>paul_swensen@norcalpublicmedia.org</t>
+          <t>bita.ryan@nbcuni.com</t>
         </is>
       </c>
       <c r="D76" s="1" t="inlineStr">
@@ -2934,7 +2934,7 @@
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>Unknown — verify in Cowork</t>
+          <t>TV news (inferred — verify)</t>
         </is>
       </c>
       <c r="G76" s="1" t="n"/>
@@ -2944,17 +2944,17 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>Jennie Butler</t>
+          <t>Velena Jones</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
         <is>
-          <t>NowThis</t>
+          <t>NBC Bay Area / NBCUniversal</t>
         </is>
       </c>
       <c r="C77" s="1" t="inlineStr">
         <is>
-          <t>jennie@nowthismedia.com</t>
+          <t>velena.jones@nbcuni.com</t>
         </is>
       </c>
       <c r="D77" s="1" t="inlineStr">
@@ -2969,23 +2969,35 @@
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>Unknown — verify in Cowork</t>
+          <t>TV news (inferred — verify)</t>
         </is>
       </c>
       <c r="G77" s="1" t="n"/>
-      <c r="H77" s="1" t="n"/>
-      <c r="I77" s="1" t="n"/>
+      <c r="H77" s="1" t="inlineStr">
+        <is>
+          <t>Typo variant nbcunic.com bounced Mar 5 — verify spelling</t>
+        </is>
+      </c>
+      <c r="I77" s="1" t="inlineStr">
+        <is>
+          <t>MED — NBC Bay Area reporter</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n"/>
+      <c r="A78" s="1" t="inlineStr">
+        <is>
+          <t>Paul Swensen</t>
+        </is>
+      </c>
       <c r="B78" s="1" t="inlineStr">
         <is>
-          <t>Oakland Observer</t>
+          <t>NorCal Public Media</t>
         </is>
       </c>
       <c r="C78" s="1" t="inlineStr">
         <is>
-          <t>oaklandobserver@hyphenatedrepublic.com</t>
+          <t>paul_swensen@norcalpublicmedia.org</t>
         </is>
       </c>
       <c r="D78" s="1" t="inlineStr">
@@ -3008,20 +3020,24 @@
       <c r="I78" s="1" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n"/>
+      <c r="A79" s="1" t="inlineStr">
+        <is>
+          <t>Jennie Butler</t>
+        </is>
+      </c>
       <c r="B79" s="1" t="inlineStr">
         <is>
-          <t>pacbell.net</t>
+          <t>NowThis</t>
         </is>
       </c>
       <c r="C79" s="1" t="inlineStr">
         <is>
-          <t>jasphoto@pacbell.net</t>
+          <t>jennie@nowthismedia.com</t>
         </is>
       </c>
       <c r="D79" s="1" t="inlineStr">
         <is>
-          <t>Photojournalist</t>
+          <t>Reporter / journalist</t>
         </is>
       </c>
       <c r="E79" s="1" t="inlineStr">
@@ -3042,17 +3058,17 @@
       <c r="A80" s="1" t="n"/>
       <c r="B80" s="1" t="inlineStr">
         <is>
-          <t>POOR Magazine</t>
+          <t>Oakland Observer</t>
         </is>
       </c>
       <c r="C80" s="1" t="inlineStr">
         <is>
-          <t>deeandtiny@poormagazine.org</t>
+          <t>oaklandobserver@hyphenatedrepublic.com</t>
         </is>
       </c>
       <c r="D80" s="1" t="inlineStr">
         <is>
-          <t>POOR Magazine (advocacy)</t>
+          <t>Reporter / journalist</t>
         </is>
       </c>
       <c r="E80" s="1" t="inlineStr">
@@ -3073,17 +3089,17 @@
       <c r="A81" s="1" t="n"/>
       <c r="B81" s="1" t="inlineStr">
         <is>
-          <t>POOR Magazine</t>
+          <t>pacbell.net</t>
         </is>
       </c>
       <c r="C81" s="1" t="inlineStr">
         <is>
-          <t>tiny@poormagazine.org</t>
+          <t>jasphoto@pacbell.net</t>
         </is>
       </c>
       <c r="D81" s="1" t="inlineStr">
         <is>
-          <t>POOR Magazine (advocacy)</t>
+          <t>Photojournalist</t>
         </is>
       </c>
       <c r="E81" s="1" t="inlineStr">
@@ -3104,17 +3120,17 @@
       <c r="A82" s="1" t="n"/>
       <c r="B82" s="1" t="inlineStr">
         <is>
-          <t>Prism</t>
+          <t>POOR Magazine</t>
         </is>
       </c>
       <c r="C82" s="1" t="inlineStr">
         <is>
-          <t>pitch@prismreports.org</t>
+          <t>deeandtiny@poormagazine.org</t>
         </is>
       </c>
       <c r="D82" s="1" t="inlineStr">
         <is>
-          <t>News desk / general</t>
+          <t>POOR Magazine (advocacy)</t>
         </is>
       </c>
       <c r="E82" s="1" t="inlineStr">
@@ -3132,24 +3148,20 @@
       <c r="I82" s="1" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="inlineStr">
-        <is>
-          <t>Josh Boswell</t>
-        </is>
-      </c>
+      <c r="A83" s="1" t="n"/>
       <c r="B83" s="1" t="inlineStr">
         <is>
-          <t>protonmail.com</t>
+          <t>POOR Magazine</t>
         </is>
       </c>
       <c r="C83" s="1" t="inlineStr">
         <is>
-          <t>josh.boswell@protonmail.com</t>
+          <t>tiny@poormagazine.org</t>
         </is>
       </c>
       <c r="D83" s="1" t="inlineStr">
         <is>
-          <t>Reporter / journalist</t>
+          <t>POOR Magazine (advocacy)</t>
         </is>
       </c>
       <c r="E83" s="1" t="inlineStr">
@@ -3167,24 +3179,20 @@
       <c r="I83" s="1" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="inlineStr">
-        <is>
-          <t>Annie Vainshtein</t>
-        </is>
-      </c>
+      <c r="A84" s="1" t="n"/>
       <c r="B84" s="1" t="inlineStr">
         <is>
-          <t>San Francisco Chronicle</t>
+          <t>Prism</t>
         </is>
       </c>
       <c r="C84" s="1" t="inlineStr">
         <is>
-          <t>avainshtein@sfchronicle.com</t>
+          <t>pitch@prismreports.org</t>
         </is>
       </c>
       <c r="D84" s="1" t="inlineStr">
         <is>
-          <t>Reporter / journalist</t>
+          <t>News desk / general</t>
         </is>
       </c>
       <c r="E84" s="1" t="inlineStr">
@@ -3194,31 +3202,27 @@
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>Metro/Bay Area news (inferred — verify)</t>
+          <t>Unknown — verify in Cowork</t>
         </is>
       </c>
       <c r="G84" s="1" t="n"/>
       <c r="H84" s="1" t="n"/>
-      <c r="I84" s="1" t="inlineStr">
-        <is>
-          <t>MED — SF Chronicle</t>
-        </is>
-      </c>
+      <c r="I84" s="1" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>Danielle Echeverria</t>
+          <t>Josh Boswell</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
         <is>
-          <t>San Francisco Chronicle</t>
+          <t>protonmail.com</t>
         </is>
       </c>
       <c r="C85" s="1" t="inlineStr">
         <is>
-          <t>danielle.echeverria@sfchronicle.com</t>
+          <t>josh.boswell@protonmail.com</t>
         </is>
       </c>
       <c r="D85" s="1" t="inlineStr">
@@ -3233,7 +3237,7 @@
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>Metro/Bay Area news (inferred — verify)</t>
+          <t>Unknown — verify in Cowork</t>
         </is>
       </c>
       <c r="G85" s="1" t="n"/>
@@ -3243,7 +3247,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>Rachel Swan</t>
+          <t>Annie Vainshtein</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3253,7 +3257,7 @@
       </c>
       <c r="C86" s="1" t="inlineStr">
         <is>
-          <t>rswan@sfchronicle.com</t>
+          <t>avainshtein@sfchronicle.com</t>
         </is>
       </c>
       <c r="D86" s="1" t="inlineStr">
@@ -3263,37 +3267,41 @@
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>ACTIVE (verified)</t>
+          <t>Not yet verified</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>Regional transportation/BART; Oakland &amp; East Bay politics</t>
+          <t>Metro/Bay Area news (inferred — verify)</t>
         </is>
       </c>
       <c r="G86" s="1" t="n"/>
       <c r="H86" s="1" t="n"/>
       <c r="I86" s="1" t="inlineStr">
         <is>
-          <t>MED — SF Chronicle, covers Oakland/East Bay</t>
+          <t>MED — SF Chronicle</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n"/>
+      <c r="A87" s="1" t="inlineStr">
+        <is>
+          <t>Danielle Echeverria</t>
+        </is>
+      </c>
       <c r="B87" s="1" t="inlineStr">
         <is>
-          <t>SF Bay View</t>
+          <t>San Francisco Chronicle</t>
         </is>
       </c>
       <c r="C87" s="1" t="inlineStr">
         <is>
-          <t>editor@sfbayview.com</t>
+          <t>danielle.echeverria@sfchronicle.com</t>
         </is>
       </c>
       <c r="D87" s="1" t="inlineStr">
         <is>
-          <t>News desk / general</t>
+          <t>Reporter / journalist</t>
         </is>
       </c>
       <c r="E87" s="1" t="inlineStr">
@@ -3303,31 +3311,27 @@
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>Black community news (inferred — verify)</t>
+          <t>Metro/Bay Area news (inferred — verify)</t>
         </is>
       </c>
       <c r="G87" s="1" t="n"/>
       <c r="H87" s="1" t="n"/>
-      <c r="I87" s="1" t="inlineStr">
-        <is>
-          <t>MED — SF Bay View (Black paper)</t>
-        </is>
-      </c>
+      <c r="I87" s="1" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>J. Lynch</t>
+          <t>Rachel Swan</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
         <is>
-          <t>SLO Tribune</t>
+          <t>San Francisco Chronicle</t>
         </is>
       </c>
       <c r="C88" s="1" t="inlineStr">
         <is>
-          <t>jlynch@thetribunenews.com</t>
+          <t>rswan@sfchronicle.com</t>
         </is>
       </c>
       <c r="D88" s="1" t="inlineStr">
@@ -3337,59 +3341,71 @@
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>Not yet verified</t>
+          <t>ACTIVE (verified)</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>Unknown — verify in Cowork</t>
+          <t>Regional transportation/BART; Oakland &amp; East Bay politics</t>
         </is>
       </c>
       <c r="G88" s="1" t="n"/>
       <c r="H88" s="1" t="n"/>
-      <c r="I88" s="1" t="n"/>
+      <c r="I88" s="1" t="inlineStr">
+        <is>
+          <t>MED — SF Chronicle, covers Oakland/East Bay</t>
+        </is>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="inlineStr">
-        <is>
-          <t>Bradley Penner</t>
-        </is>
-      </c>
+      <c r="A89" s="1" t="n"/>
       <c r="B89" s="1" t="inlineStr">
         <is>
-          <t>Street Spirit</t>
-        </is>
-      </c>
-      <c r="C89" s="1" t="n"/>
+          <t>SF Bay View</t>
+        </is>
+      </c>
+      <c r="C89" s="1" t="inlineStr">
+        <is>
+          <t>editor@sfbayview.com</t>
+        </is>
+      </c>
       <c r="D89" s="1" t="inlineStr">
         <is>
-          <t>Reporter / journalist</t>
+          <t>News desk / general</t>
         </is>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>auto-added from byline — needs contact info</t>
-        </is>
-      </c>
-      <c r="F89" s="1" t="n"/>
+          <t>Not yet verified</t>
+        </is>
+      </c>
+      <c r="F89" s="1" t="inlineStr">
+        <is>
+          <t>Black community news (inferred — verify)</t>
+        </is>
+      </c>
       <c r="G89" s="1" t="n"/>
       <c r="H89" s="1" t="n"/>
-      <c r="I89" s="1" t="n"/>
+      <c r="I89" s="1" t="inlineStr">
+        <is>
+          <t>MED — SF Bay View (Black paper)</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>G. Lang</t>
+          <t>J. Lynch</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
         <is>
-          <t>The Ark / Marinscope</t>
+          <t>SLO Tribune</t>
         </is>
       </c>
       <c r="C90" s="1" t="inlineStr">
         <is>
-          <t>glang@thearknewspaper.com</t>
+          <t>jlynch@thetribunenews.com</t>
         </is>
       </c>
       <c r="D90" s="1" t="inlineStr">
@@ -3404,7 +3420,7 @@
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>Southern Marin community news (inferred — verify)</t>
+          <t>Unknown — verify in Cowork</t>
         </is>
       </c>
       <c r="G90" s="1" t="n"/>
@@ -3412,32 +3428,28 @@
       <c r="I90" s="1" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n"/>
+      <c r="A91" s="1" t="inlineStr">
+        <is>
+          <t>Bradley Penner</t>
+        </is>
+      </c>
       <c r="B91" s="1" t="inlineStr">
         <is>
-          <t>The Ark / Marinscope</t>
-        </is>
-      </c>
-      <c r="C91" s="1" t="inlineStr">
-        <is>
-          <t>editor@thearknewspaper.com</t>
-        </is>
-      </c>
+          <t>Street Spirit</t>
+        </is>
+      </c>
+      <c r="C91" s="1" t="n"/>
       <c r="D91" s="1" t="inlineStr">
         <is>
-          <t>News desk / general</t>
+          <t>Reporter / journalist</t>
         </is>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>Not yet verified</t>
-        </is>
-      </c>
-      <c r="F91" s="1" t="inlineStr">
-        <is>
-          <t>Southern Marin community news (inferred — verify)</t>
-        </is>
-      </c>
+          <t>auto-added from byline — needs contact info</t>
+        </is>
+      </c>
+      <c r="F91" s="1" t="n"/>
       <c r="G91" s="1" t="n"/>
       <c r="H91" s="1" t="n"/>
       <c r="I91" s="1" t="n"/>
@@ -3445,17 +3457,17 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>Esme Hyatt</t>
+          <t>G. Lang</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
         <is>
-          <t>The Daily Californian</t>
+          <t>The Ark / Marinscope</t>
         </is>
       </c>
       <c r="C92" s="1" t="inlineStr">
         <is>
-          <t>ehyatt@dailycal.org</t>
+          <t>glang@thearknewspaper.com</t>
         </is>
       </c>
       <c r="D92" s="1" t="inlineStr">
@@ -3470,7 +3482,7 @@
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>UC Berkeley &amp; city news; encampments/housing</t>
+          <t>Southern Marin community news (inferred — verify)</t>
         </is>
       </c>
       <c r="G92" s="1" t="n"/>
@@ -3481,12 +3493,12 @@
       <c r="A93" s="1" t="n"/>
       <c r="B93" s="1" t="inlineStr">
         <is>
-          <t>The Daily Californian</t>
+          <t>The Ark / Marinscope</t>
         </is>
       </c>
       <c r="C93" s="1" t="inlineStr">
         <is>
-          <t>editor@dailycal.org</t>
+          <t>editor@thearknewspaper.com</t>
         </is>
       </c>
       <c r="D93" s="1" t="inlineStr">
@@ -3501,7 +3513,7 @@
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>UC Berkeley student paper (inferred — verify)</t>
+          <t>Southern Marin community news (inferred — verify)</t>
         </is>
       </c>
       <c r="G93" s="1" t="n"/>
@@ -3511,17 +3523,17 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>Lois Beckett</t>
+          <t>Esme Hyatt</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
         <is>
-          <t>The Guardian (US)</t>
+          <t>The Daily Californian</t>
         </is>
       </c>
       <c r="C94" s="1" t="inlineStr">
         <is>
-          <t>lois.beckett@theguardian.com</t>
+          <t>ehyatt@dailycal.org</t>
         </is>
       </c>
       <c r="D94" s="1" t="inlineStr">
@@ -3536,7 +3548,7 @@
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>Guns, far-right, California (Guardian US)</t>
+          <t>UC Berkeley &amp; city news; encampments/housing</t>
         </is>
       </c>
       <c r="G94" s="1" t="n"/>
@@ -3544,24 +3556,20 @@
       <c r="I94" s="1" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="inlineStr">
-        <is>
-          <t>Shawn Hubler</t>
-        </is>
-      </c>
+      <c r="A95" s="1" t="n"/>
       <c r="B95" s="1" t="inlineStr">
         <is>
-          <t>The New York Times</t>
+          <t>The Daily Californian</t>
         </is>
       </c>
       <c r="C95" s="1" t="inlineStr">
         <is>
-          <t>shawn.hubler@nytimes.com</t>
+          <t>editor@dailycal.org</t>
         </is>
       </c>
       <c r="D95" s="1" t="inlineStr">
         <is>
-          <t>Reporter / journalist</t>
+          <t>News desk / general</t>
         </is>
       </c>
       <c r="E95" s="1" t="inlineStr">
@@ -3571,7 +3579,7 @@
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>National/California news (inferred — verify)</t>
+          <t>UC Berkeley student paper (inferred — verify)</t>
         </is>
       </c>
       <c r="G95" s="1" t="n"/>
@@ -3581,17 +3589,17 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>Darwin BondGraham</t>
+          <t>Lois Beckett</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
         <is>
-          <t>The Oaklandside</t>
+          <t>The Guardian (US)</t>
         </is>
       </c>
       <c r="C96" s="1" t="inlineStr">
         <is>
-          <t>darwin@oaklandside.org</t>
+          <t>lois.beckett@theguardian.com</t>
         </is>
       </c>
       <c r="D96" s="1" t="inlineStr">
@@ -3606,31 +3614,27 @@
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>Policing, OPD, use-of-force, public records, investigations</t>
+          <t>Guns, far-right, California (Guardian US)</t>
         </is>
       </c>
       <c r="G96" s="1" t="n"/>
       <c r="H96" s="1" t="n"/>
-      <c r="I96" s="1" t="inlineStr">
-        <is>
-          <t>HIGH — Oaklandside leads OPD/records coverage</t>
-        </is>
-      </c>
+      <c r="I96" s="1" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>Andrew Graham</t>
+          <t>Shawn Hubler</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
         <is>
-          <t>The Press Democrat</t>
+          <t>The New York Times</t>
         </is>
       </c>
       <c r="C97" s="1" t="inlineStr">
         <is>
-          <t>andrew.graham@pressdemocrat.com</t>
+          <t>shawn.hubler@nytimes.com</t>
         </is>
       </c>
       <c r="D97" s="1" t="inlineStr">
@@ -3645,7 +3649,7 @@
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>North Bay/Sonoma news (inferred — verify)</t>
+          <t>National/California news (inferred — verify)</t>
         </is>
       </c>
       <c r="G97" s="1" t="n"/>
@@ -3653,20 +3657,24 @@
       <c r="I97" s="1" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n"/>
+      <c r="A98" s="1" t="inlineStr">
+        <is>
+          <t>Darwin BondGraham</t>
+        </is>
+      </c>
       <c r="B98" s="1" t="inlineStr">
         <is>
-          <t>The Progressive</t>
+          <t>The Oaklandside</t>
         </is>
       </c>
       <c r="C98" s="1" t="inlineStr">
         <is>
-          <t>editorial@progressive.org</t>
+          <t>darwin@oaklandside.org</t>
         </is>
       </c>
       <c r="D98" s="1" t="inlineStr">
         <is>
-          <t>News desk / general</t>
+          <t>Reporter / journalist</t>
         </is>
       </c>
       <c r="E98" s="1" t="inlineStr">
@@ -3676,27 +3684,31 @@
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>Unknown — verify in Cowork</t>
+          <t>Policing, OPD, use-of-force, public records, investigations</t>
         </is>
       </c>
       <c r="G98" s="1" t="n"/>
       <c r="H98" s="1" t="n"/>
-      <c r="I98" s="1" t="n"/>
+      <c r="I98" s="1" t="inlineStr">
+        <is>
+          <t>HIGH — Oaklandside leads OPD/records coverage</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>R. Byer</t>
+          <t>Andrew Graham</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
         <is>
-          <t>The Sacramento Bee</t>
+          <t>The Press Democrat</t>
         </is>
       </c>
       <c r="C99" s="1" t="inlineStr">
         <is>
-          <t>rbyer@sacbee.com</t>
+          <t>andrew.graham@pressdemocrat.com</t>
         </is>
       </c>
       <c r="D99" s="1" t="inlineStr">
@@ -3711,7 +3723,7 @@
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>Sacramento news (inferred — verify)</t>
+          <t>North Bay/Sonoma news (inferred — verify)</t>
         </is>
       </c>
       <c r="G99" s="1" t="n"/>
@@ -3719,24 +3731,20 @@
       <c r="I99" s="1" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="inlineStr">
-        <is>
-          <t>David (SF Standard)</t>
-        </is>
-      </c>
+      <c r="A100" s="1" t="n"/>
       <c r="B100" s="1" t="inlineStr">
         <is>
-          <t>The San Francisco Standard</t>
+          <t>The Progressive</t>
         </is>
       </c>
       <c r="C100" s="1" t="inlineStr">
         <is>
-          <t>david@sfstandard.com</t>
+          <t>editorial@progressive.org</t>
         </is>
       </c>
       <c r="D100" s="1" t="inlineStr">
         <is>
-          <t>Reporter / journalist</t>
+          <t>News desk / general</t>
         </is>
       </c>
       <c r="E100" s="1" t="inlineStr">
@@ -3746,31 +3754,27 @@
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>SF news (inferred — verify)</t>
+          <t>Unknown — verify in Cowork</t>
         </is>
       </c>
       <c r="G100" s="1" t="n"/>
       <c r="H100" s="1" t="n"/>
-      <c r="I100" s="1" t="inlineStr">
-        <is>
-          <t>MED — SF Standard</t>
-        </is>
-      </c>
+      <c r="I100" s="1" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>Danny Fortson</t>
+          <t>R. Byer</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
         <is>
-          <t>The Sunday Times (UK)</t>
+          <t>The Sacramento Bee</t>
         </is>
       </c>
       <c r="C101" s="1" t="inlineStr">
         <is>
-          <t>danny.fortson@sunday-times.co.uk</t>
+          <t>rbyer@sacbee.com</t>
         </is>
       </c>
       <c r="D101" s="1" t="inlineStr">
@@ -3785,7 +3789,7 @@
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>Unknown — verify in Cowork</t>
+          <t>Sacramento news (inferred — verify)</t>
         </is>
       </c>
       <c r="G101" s="1" t="n"/>
@@ -3795,17 +3799,17 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>Lisa Gartner</t>
+          <t>David (SF Standard)</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
         <is>
-          <t>The Washington Post</t>
+          <t>The San Francisco Standard</t>
         </is>
       </c>
       <c r="C102" s="1" t="inlineStr">
         <is>
-          <t>lisa.gartner@washpost.com</t>
+          <t>david@sfstandard.com</t>
         </is>
       </c>
       <c r="D102" s="1" t="inlineStr">
@@ -3820,23 +3824,31 @@
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>National news (inferred — verify)</t>
+          <t>SF news (inferred — verify)</t>
         </is>
       </c>
       <c r="G102" s="1" t="n"/>
       <c r="H102" s="1" t="n"/>
-      <c r="I102" s="1" t="n"/>
+      <c r="I102" s="1" t="inlineStr">
+        <is>
+          <t>MED — SF Standard</t>
+        </is>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n"/>
+      <c r="A103" s="1" t="inlineStr">
+        <is>
+          <t>Danny Fortson</t>
+        </is>
+      </c>
       <c r="B103" s="1" t="inlineStr">
         <is>
-          <t>tmmdl.com</t>
+          <t>The Sunday Times (UK)</t>
         </is>
       </c>
       <c r="C103" s="1" t="inlineStr">
         <is>
-          <t>neal@tmmdl.com</t>
+          <t>danny.fortson@sunday-times.co.uk</t>
         </is>
       </c>
       <c r="D103" s="1" t="inlineStr">
@@ -3859,20 +3871,24 @@
       <c r="I103" s="1" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n"/>
+      <c r="A104" s="1" t="inlineStr">
+        <is>
+          <t>Lisa Gartner</t>
+        </is>
+      </c>
       <c r="B104" s="1" t="inlineStr">
         <is>
-          <t>Truthout</t>
+          <t>The Washington Post</t>
         </is>
       </c>
       <c r="C104" s="1" t="inlineStr">
         <is>
-          <t>info@truthout.org</t>
+          <t>lisa.gartner@washpost.com</t>
         </is>
       </c>
       <c r="D104" s="1" t="inlineStr">
         <is>
-          <t>News desk / general</t>
+          <t>Reporter / journalist</t>
         </is>
       </c>
       <c r="E104" s="1" t="inlineStr">
@@ -3882,7 +3898,7 @@
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>Unknown — verify in Cowork</t>
+          <t>National news (inferred — verify)</t>
         </is>
       </c>
       <c r="G104" s="1" t="n"/>
@@ -3890,19 +3906,15 @@
       <c r="I104" s="1" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="inlineStr">
-        <is>
-          <t>Marco della Cava</t>
-        </is>
-      </c>
+      <c r="A105" s="1" t="n"/>
       <c r="B105" s="1" t="inlineStr">
         <is>
-          <t>USA Today</t>
+          <t>tmmdl.com</t>
         </is>
       </c>
       <c r="C105" s="1" t="inlineStr">
         <is>
-          <t>mdellaca@usatoday.com</t>
+          <t>neal@tmmdl.com</t>
         </is>
       </c>
       <c r="D105" s="1" t="inlineStr">
@@ -3917,7 +3929,7 @@
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>National features (inferred — verify)</t>
+          <t>Unknown — verify in Cowork</t>
         </is>
       </c>
       <c r="G105" s="1" t="n"/>
@@ -3928,17 +3940,17 @@
       <c r="A106" s="1" t="n"/>
       <c r="B106" s="1" t="inlineStr">
         <is>
-          <t>wdwg.org</t>
+          <t>Truthout</t>
         </is>
       </c>
       <c r="C106" s="1" t="inlineStr">
         <is>
-          <t>advocacy@wdwg.org</t>
+          <t>info@truthout.org</t>
         </is>
       </c>
       <c r="D106" s="1" t="inlineStr">
         <is>
-          <t>Advocacy — WDWG</t>
+          <t>News desk / general</t>
         </is>
       </c>
       <c r="E106" s="1" t="inlineStr">
@@ -3958,22 +3970,22 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>Paul Boden</t>
+          <t>Marco della Cava</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
         <is>
-          <t>wraphome.org</t>
+          <t>USA Today</t>
         </is>
       </c>
       <c r="C107" s="1" t="inlineStr">
         <is>
-          <t>pboden@wraphome.org</t>
+          <t>mdellaca@usatoday.com</t>
         </is>
       </c>
       <c r="D107" s="1" t="inlineStr">
         <is>
-          <t>Advocacy — WRAP</t>
+          <t>Reporter / journalist</t>
         </is>
       </c>
       <c r="E107" s="1" t="inlineStr">
@@ -3983,7 +3995,7 @@
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>Unknown — verify in Cowork</t>
+          <t>National features (inferred — verify)</t>
         </is>
       </c>
       <c r="G107" s="1" t="n"/>
@@ -3991,24 +4003,20 @@
       <c r="I107" s="1" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="inlineStr">
-        <is>
-          <t>Nikki Silverstein</t>
-        </is>
-      </c>
+      <c r="A108" s="1" t="n"/>
       <c r="B108" s="1" t="inlineStr">
         <is>
-          <t>yahoo.com</t>
+          <t>wdwg.org</t>
         </is>
       </c>
       <c r="C108" s="1" t="inlineStr">
         <is>
-          <t>nikki_silverstein@yahoo.com</t>
+          <t>advocacy@wdwg.org</t>
         </is>
       </c>
       <c r="D108" s="1" t="inlineStr">
         <is>
-          <t>Reporter / journalist</t>
+          <t>Advocacy — WDWG</t>
         </is>
       </c>
       <c r="E108" s="1" t="inlineStr">
@@ -4026,20 +4034,24 @@
       <c r="I108" s="1" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n"/>
+      <c r="A109" s="1" t="inlineStr">
+        <is>
+          <t>Paul Boden</t>
+        </is>
+      </c>
       <c r="B109" s="1" t="inlineStr">
         <is>
-          <t>yahoo.com</t>
+          <t>wraphome.org</t>
         </is>
       </c>
       <c r="C109" s="1" t="inlineStr">
         <is>
-          <t>webike@yahoo.com</t>
+          <t>pboden@wraphome.org</t>
         </is>
       </c>
       <c r="D109" s="1" t="inlineStr">
         <is>
-          <t>Reporter / journalist</t>
+          <t>Advocacy — WRAP</t>
         </is>
       </c>
       <c r="E109" s="1" t="inlineStr">
@@ -4057,7 +4069,11 @@
       <c r="I109" s="1" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n"/>
+      <c r="A110" s="1" t="inlineStr">
+        <is>
+          <t>Nikki Silverstein</t>
+        </is>
+      </c>
       <c r="B110" s="1" t="inlineStr">
         <is>
           <t>yahoo.com</t>
@@ -4065,12 +4081,12 @@
       </c>
       <c r="C110" s="1" t="inlineStr">
         <is>
-          <t>berkeleycopwatch@yahoo.com</t>
+          <t>nikki_silverstein@yahoo.com</t>
         </is>
       </c>
       <c r="D110" s="1" t="inlineStr">
         <is>
-          <t>Advocacy — Copwatch</t>
+          <t>Reporter / journalist</t>
         </is>
       </c>
       <c r="E110" s="1" t="inlineStr">
@@ -4096,12 +4112,12 @@
       </c>
       <c r="C111" s="1" t="inlineStr">
         <is>
-          <t>princelawoffices@yahoo.com</t>
+          <t>webike@yahoo.com</t>
         </is>
       </c>
       <c r="D111" s="1" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Reporter / journalist</t>
         </is>
       </c>
       <c r="E111" s="1" t="inlineStr">
@@ -4117,6 +4133,68 @@
       <c r="G111" s="1" t="n"/>
       <c r="H111" s="1" t="n"/>
       <c r="I111" s="1" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="n"/>
+      <c r="B112" s="1" t="inlineStr">
+        <is>
+          <t>yahoo.com</t>
+        </is>
+      </c>
+      <c r="C112" s="1" t="inlineStr">
+        <is>
+          <t>berkeleycopwatch@yahoo.com</t>
+        </is>
+      </c>
+      <c r="D112" s="1" t="inlineStr">
+        <is>
+          <t>Advocacy — Copwatch</t>
+        </is>
+      </c>
+      <c r="E112" s="1" t="inlineStr">
+        <is>
+          <t>Not yet verified</t>
+        </is>
+      </c>
+      <c r="F112" s="1" t="inlineStr">
+        <is>
+          <t>Unknown — verify in Cowork</t>
+        </is>
+      </c>
+      <c r="G112" s="1" t="n"/>
+      <c r="H112" s="1" t="n"/>
+      <c r="I112" s="1" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="1" t="n"/>
+      <c r="B113" s="1" t="inlineStr">
+        <is>
+          <t>yahoo.com</t>
+        </is>
+      </c>
+      <c r="C113" s="1" t="inlineStr">
+        <is>
+          <t>princelawoffices@yahoo.com</t>
+        </is>
+      </c>
+      <c r="D113" s="1" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="E113" s="1" t="inlineStr">
+        <is>
+          <t>Not yet verified</t>
+        </is>
+      </c>
+      <c r="F113" s="1" t="inlineStr">
+        <is>
+          <t>Unknown — verify in Cowork</t>
+        </is>
+      </c>
+      <c r="G113" s="1" t="n"/>
+      <c r="H113" s="1" t="n"/>
+      <c r="I113" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4132,11 +4210,11 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>

</xml_diff>